<commit_message>
minor updatre to fix wierd problem with Rules
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B02A5222-A645-4F8C-BC6A-D4505F0B22F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFD65D27-4847-4793-A66C-9EE1C5E3109E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -33,7 +33,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>e001</t>
+  </si>
   <si>
     <t>e000</t>
   </si>
@@ -68,6 +71,16 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
+    <t>&lt;Bold&gt;e001 Secretly Select HQ Area&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
+The first step is for the Alien player to secretly choose where the Alien Sub-Commander is running his operations.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The headquarters (HQ) must be a specified building, such as &lt;Bold&gt;House 4&lt;/Bold&gt; the &lt;Bold&gt;Stock Pen&lt;/Bold&gt; , the &lt;Bold&gt;Town Hall&lt;/Bold&gt;, etc. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If the building chosen as the Alien HQ has more than one space, the Alien player must choose which area of the building is the Alien HQ. This information is secret to the Alien Player.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                            &lt;InlineUIContainer&gt;&lt;Image Name='ZebulonBlack'  Height='150' Width='150'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
     <t>&lt;Bold&gt;e000 Game Introduction&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
 &lt;Bold&gt;They&amp;apos;ve Invaded Pleasantville&lt;/Bold&gt; minigame is a two-player game of a secret invasion by space aliens.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -77,16 +90,16 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Choose a button to begin:
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Name='ReadRules' Content=' Read Rules ' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;InlineUIContainer&gt;&lt;Button Name='ReadRules' Content=' Read Rules ' FontFamily='Courier New'  FontSize='12' IsEnabled='False'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Rules presented as needed if choose to skip&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Name='HostGame' Content=' Host Game  ' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Host a game on your computer &lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Name='JoinGame' Content=' Join Game  ' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
- - join a game somebody is hosting&lt;LineBreak/&gt;
+ - Join a game somebody is hosting&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Name='PlayTown' Content=' Town Solo  ' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
- - play as the Townsplayer against computer&lt;LineBreak/&gt;
+ - Play as the Townsplayer against computer&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Name='PlayAlien' Content=' Alien Solo ' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
- - play as Alien against computer&lt;LineBreak/&gt;</t>
+ - Play as Alien against computer&lt;LineBreak/&gt;</t>
   </si>
 </sst>
 </file>
@@ -450,7 +463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -459,18 +472,18 @@
   <sheetData>
     <row r="1" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -483,18 +496,26 @@
     </row>
     <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
     </row>
-    <row r="5" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added behavior to move and drop map items
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{92080143-7ACD-441A-9488-C515410F49B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AFF0889-0FD5-4EE8-B746-ECC49228CB5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -71,6 +71,17 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
+    <t>&lt;Bold&gt;e001 Secretly Select HQ Area&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r3.1' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
+The first step is for the Alien player to secretly choose where the Alien Sub-Commander is running his operations.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The headquarters (HQ) must be a specified building, such as &lt;Bold&gt;House 4&lt;/Bold&gt; the &lt;Bold&gt;Stock Pen&lt;/Bold&gt; , the &lt;Bold&gt;Town Hall&lt;/Bold&gt;, etc. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If the building chosen as the Alien HQ has more than one space, the Alien player must choose which area of the building is the Alien HQ. This information is secret to the Alien Player.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                            &lt;InlineUIContainer&gt;&lt;Image Name='ZebulonBlack'  Height='150' Width='150'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
     <t>&lt;Bold&gt;e000 Game Introduction&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
 &lt;Bold&gt;They&amp;apos;ve Invaded Pleasantville&lt;/Bold&gt; minigame is a two-player game of a secret invasion by space aliens.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -82,25 +93,14 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Name='ReadRules' Content=' Read Rules ' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Rules presented as needed if choose to skip&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Name='HostGame' Content=' Host Game  ' FontFamily='Courier New'  FontSize='12'  IsEnabled='False'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;InlineUIContainer&gt;&lt;Button Name='HostGame' Content=' Host Game  ' FontFamily='Courier New'  FontSize='12'  &gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Host a game on your computer &lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Name='JoinGame' Content=' Join Game  ' FontFamily='Courier New'  FontSize='12'  IsEnabled='False'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;InlineUIContainer&gt;&lt;Button Name='JoinGame' Content=' Join Game  ' FontFamily='Courier New'  FontSize='12'  &gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Join a game somebody is hosting&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Name='PlayTown' Content=' Town Solo  ' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Play as the Townsplayer against computer&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Name='PlayAlien' Content=' Alien Solo ' FontFamily='Courier New'  FontSize='12'  IsEnabled='False'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;InlineUIContainer&gt;&lt;Button Name='PlayAlien' Content=' Alien Solo ' FontFamily='Courier New'  FontSize='12'  &gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Play as Alien against computer&lt;LineBreak/&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e001 Secretly Select HQ Area&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r3.1' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
-The first step is for the Alien player to secretly choose where the Alien Sub-Commander is running his operations.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The headquarters (HQ) must be a specified building, such as &lt;Bold&gt;House 4&lt;/Bold&gt; the &lt;Bold&gt;Stock Pen&lt;/Bold&gt; , the &lt;Bold&gt;Town Hall&lt;/Bold&gt;, etc. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-If the building chosen as the Alien HQ has more than one space, the Alien player must choose which area of the building is the Alien HQ. This information is secret to the Alien Player.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                            &lt;InlineUIContainer&gt;&lt;Image Name='ZebulonBlack'  Height='150' Width='150'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -476,7 +476,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -484,7 +484,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
started adding starting alien player
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE0D1A8D-9626-4C20-9282-7A390A17D420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{251619CB-8F97-4730-AC4A-0EB216A4B045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>e001</t>
   </si>
@@ -110,6 +110,17 @@
 If the building chosen as the Alien HQ has more than one space, the Alien player must choose which area of the building is the Alien HQ. This information is secret to the Alien Player.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                             &lt;InlineUIContainer&gt;&lt;Image Name='ZebulonBlack'  Height='150' Width='150'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e003</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e003 Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Alien player secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
+to determine which two townspersons begin the game under Alien control. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Alien player cannot begin with the same character as the Town player. Such a result requires rerolling the die to get a different result. Also, note that any 1st die roll of 6 must be rerolled when using this table.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
 </sst>
 </file>
@@ -473,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -504,35 +515,43 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
working next stage of preps
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE0D1A8D-9626-4C20-9282-7A390A17D420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC82BF78-EDE1-47D4-BD1A-94E5E54E19CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>e001</t>
   </si>
@@ -110,6 +110,25 @@
 If the building chosen as the Alien HQ has more than one space, the Alien player must choose which area of the building is the Alien HQ. This information is secret to the Alien Player.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                             &lt;InlineUIContainer&gt;&lt;Image Name='ZebulonBlack'  Height='150' Width='150'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e003</t>
+  </si>
+  <si>
+    <t>e003a</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e003 Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Alien player secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
+to determine which two townspersons begin the game under Alien control. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e003a Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The computer secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
+to determine which two townspersons begin the game under Alien control. This information is hidden from Towns player.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                            &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -473,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -504,35 +523,51 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="9" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
working thru setup issues
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC82BF78-EDE1-47D4-BD1A-94E5E54E19CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{40C0B700-EC2E-418D-8266-D4602AA1DAF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>e001</t>
   </si>
@@ -126,9 +126,33 @@
   <si>
     <t>&lt;Bold&gt;e003a Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
 The computer secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
-to determine which two townspersons begin the game under Alien control. This information is hidden from Towns player.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                            &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+to determine which two townspersons begin the game under Alien control. This information is hidden from Towns player. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                  &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e004</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e004 Setting Up Map&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The starting locations for each piece is printed in the upper-left of the corner of the counter per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Every counter is placed on the map.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If a building has more than one space in it, the counter is placed randomly in one of the spaces. However, only one counter may be placed in each space. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The starting townplayer is shown in green. The alien is only one to see starting aliens until they become known. They are showed in gold. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                  &lt;InlineUIContainer&gt;&lt;Image Name='Continue004' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e005</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e005 Random Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Four townspeople (if not under Town player control) move randomly in any given turn. The &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines who moves. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The destination is per the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Target Building' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table.</t>
   </si>
 </sst>
 </file>
@@ -492,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -539,35 +563,51 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="11" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Got initial random move selection working
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40C0B700-EC2E-418D-8266-D4602AA1DAF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF287034-C2DD-4854-9C77-AD1975261707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -151,8 +151,14 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Four townspeople (if not under Town player control) move randomly in any given turn. The &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines who moves. 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Tied Up, Unconscious, Killed players do not move. Only move a townsperson once. Stunned counters still move. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If a controlled townsperson (either Town or Alien) is moved, the owner has the option to not move. However, if the alien player, this exposes the unknown alien. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
 The destination is per the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Target Building' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table.</t>
+&lt;InlineUIContainer&gt;&lt;Button Content='Target Building' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                  &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -571,7 +577,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
Updated to do Random Moves outside of EventViewer
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\Documents\HereWeGo\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF287034-C2DD-4854-9C77-AD1975261707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{766CBD19-AC28-4501-983F-BF6126E49A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -101,17 +101,6 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e001 Secretly Select HQ Area&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r3.1' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
-The Alien player secretly chooses where the Alien Sub-Commander is running his operations.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The headquarters (HQ) must be a specified building, such as &lt;Bold&gt;House 4&lt;/Bold&gt; the &lt;Bold&gt;Stock Pen&lt;/Bold&gt; , the &lt;Bold&gt;Town Hall&lt;/Bold&gt;, etc. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-If the building chosen as the Alien HQ has more than one space, the Alien player must choose which area of the building is the Alien HQ. This information is secret to the Alien Player.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                            &lt;InlineUIContainer&gt;&lt;Image Name='ZebulonBlack'  Height='150' Width='150'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
     <t>e003</t>
   </si>
   <si>
@@ -124,14 +113,40 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
+    <t>e004</t>
+  </si>
+  <si>
+    <t>e005</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e001 Secretly Select HQ Area&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r3.1' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
+The Alien player secretly chooses where the Alien Sub-Commander is running his operations.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The headquarters (HQ) must be a specified building, such as &lt;Bold&gt;House 4&lt;/Bold&gt; the &lt;Bold&gt;Stock Pen&lt;/Bold&gt; , the &lt;Bold&gt;Town Hall&lt;/Bold&gt;, etc. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If the building chosen as the Alien HQ has more than one space, the Alien player must choose which area of the building is the Alien HQ. This information is secret to the Alien Player.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                       &lt;InlineUIContainer&gt;&lt;Image Name='ZebulonBlack'  Height='150' Width='150'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
     <t>&lt;Bold&gt;e003a Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
 The computer secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
 to determine which two townspersons begin the game under Alien control. This information is hidden from Towns player. Click image to continue.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                  &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>e004</t>
+                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e005 Random Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Four townspeople move randomly in any given turn. The &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines who moves. The destination is per the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Target Building' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Tied-up, Unconscious, or Killed people do not move. Stunned still move.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If a controlled townsperson (either Town or Alien) is moved, the owner has the option to not move. However, the Alien player exposes that it is an alien controlled person if not known. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
     <t>&lt;Bold&gt;e004 Setting Up Map&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -139,26 +154,9 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 If a building has more than one space in it, the counter is placed randomly in one of the spaces. However, only one counter may be placed in each space. 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The starting townplayer is shown in green. The alien is only one to see starting aliens until they become known. They are showed in gold. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                  &lt;InlineUIContainer&gt;&lt;Image Name='Continue004' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>e005</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e005 Random Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Four townspeople (if not under Town player control) move randomly in any given turn. The &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines who moves. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Tied Up, Unconscious, Killed players do not move. Only move a townsperson once. Stunned counters still move. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-If a controlled townsperson (either Town or Alien) is moved, the owner has the option to not move. However, if the alien player, this exposes the unknown alien. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The destination is per the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Target Building' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                  &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+The starting Town's controlled townsperson is shown in green. The Alien player is only one to see starting aliens until they become known. They are showed in gold. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue004' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -542,7 +540,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -555,34 +553,34 @@
     </row>
     <row r="4" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="195" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
adding finding map path for random move
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\Documents\HereWeGo\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{766CBD19-AC28-4501-983F-BF6126E49A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB7D331C-653D-47D9-AC20-80CEB570D391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -137,6 +137,16 @@
                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
+    <t>&lt;Bold&gt;e004 Setting Up Map&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The starting locations for each piece is printed in the upper-left of the corner of the counter per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Every counter is placed on the map.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If a building has more than one space in it, the counter is placed randomly in one of the spaces. However, only one counter may be placed in each space. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The starting Town's controlled townsperson is shown in green. The Alien player is only one to see starting aliens until they become known. They are showed in gold. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue004' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
     <t>&lt;Bold&gt;e005 Random Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Four townspeople move randomly in any given turn. The &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines who moves. The destination is per the 
@@ -144,19 +154,9 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Tied-up, Unconscious, or Killed people do not move. Stunned still move.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-If a controlled townsperson (either Town or Alien) is moved, the owner has the option to not move. However, the Alien player exposes that it is an alien controlled person if not known. Click image to continue.
+If a controlled townsperson (either Town or Alien) is selected, the owner has the option to block moving it. However, the Alien player exposes that it is an alien controlled person if not known. Click image to continue.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e004 Setting Up Map&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The starting locations for each piece is printed in the upper-left of the corner of the counter per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Every counter is placed on the map.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-If a building has more than one space in it, the counter is placed randomly in one of the spaces. However, only one counter may be placed in each space. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The starting Town's controlled townsperson is shown in green. The Alien player is only one to see starting aliens until they become known. They are showed in gold. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue004' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -572,7 +572,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -580,7 +580,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
trying to work on logic for muliple playsers
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\Documents\HereWeGo\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB7D331C-653D-47D9-AC20-80CEB570D391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F873FFD-4B99-4426-8092-C1A26AD26805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>e001</t>
   </si>
@@ -157,6 +157,63 @@
 If a controlled townsperson (either Town or Alien) is selected, the owner has the option to block moving it. However, the Alien player exposes that it is an alien controlled person if not known. Click image to continue.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e006a</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e006 Alien Player Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+During his or her movement phase, the Alien player may move up to five townsperson counters. However, these townspeople may not be:
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Controlled by Town player per &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Wary per &lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables&lt;LineBreak/&gt;
+-- Stunned per &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+In effect, the Alien player is limited to moving up to five counters that are either Alien controlled, skeptical per 
+&lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
+or totally uncontrolled. Click an uncontrolled or controlled skeptical counter to move. Select their destination. They move up to their maximum movement allowance &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. You can select intermediate way points to move in a more controlled path.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click image below to continue when done moving all counters.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e005a</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e005a Awaiting Alien Confirmation of Random Move&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Alien player needs to confirm random moves before continuing.</t>
+  </si>
+  <si>
+    <t>e005t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e005t Awaiting Town Confirmation of Random Move&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Town player needs to confirm random moves before continuing.</t>
+  </si>
+  <si>
+    <t>e006t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e006t Alien Player Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+During his or her movement phase, the Alien player may move up to five townsperson counters. However, these townspeople may not be:
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Controlled by Town player per &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Wary per &lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables&lt;LineBreak/&gt;
+-- Stunned per &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+In effect, the Alien player is limited to moving up to five counters that are either Alien controlled, skeptical per 
+&lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
+or totally uncontrolled. Since you are the Townsplayer, you are waiting for that to happen.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
 </sst>
 </file>
@@ -520,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -583,35 +640,67 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="285" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="225" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="13" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="15" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
working toward random moves
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\Documents\HereWeGo\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F873FFD-4B99-4426-8092-C1A26AD26805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D88A6955-2059-4777-931A-3BA4E5B19F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-23670" yWindow="1905" windowWidth="21600" windowHeight="11295" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -101,16 +101,7 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
-    <t>e003</t>
-  </si>
-  <si>
     <t>e003a</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e003 Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Alien player secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
-to determine which two townspersons begin the game under Alien control. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
     <t>e004</t>
@@ -128,13 +119,6 @@
 If the building chosen as the Alien HQ has more than one space, the Alien player must choose which area of the building is the Alien HQ. This information is secret to the Alien Player.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                        &lt;InlineUIContainer&gt;&lt;Image Name='ZebulonBlack'  Height='150' Width='150'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e003a Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The computer secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
-to determine which two townspersons begin the game under Alien control. This information is hidden from Towns player. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
     <t>&lt;Bold&gt;e004 Setting Up Map&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -214,6 +198,22 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
 or totally uncontrolled. Since you are the Townsplayer, you are waiting for that to happen.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>e003t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e003a Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Alien player secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
+to determine which two townspersons begin the game under Alien control. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e003t Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The computer secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
+to determine which two townspersons begin the game under Alien control. This information is hidden from Towns player. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -613,63 +613,63 @@
         <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="225" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Moving to alien movement
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\Documents\HereWeGo\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D88A6955-2059-4777-931A-3BA4E5B19F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6CAD835-0B15-4E4E-B150-443C2C5FE372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23670" yWindow="1905" windowWidth="21600" windowHeight="11295" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -176,17 +176,35 @@
     <t>e005t</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e005t Awaiting Town Confirmation of Random Move&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Town player needs to confirm random moves before continuing.</t>
-  </si>
-  <si>
     <t>e006t</t>
   </si>
   <si>
+    <t>e003t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e003a Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Alien player secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
+to determine which two townspersons begin the game under Alien control. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e003t Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The computer secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
+to determine which two townspersons begin the game under Alien control. This information is hidden from Towns player. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e005t Confirm Random Move&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Confirm random moves by clicking image.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
     <t>&lt;Bold&gt;e006t Alien Player Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-During his or her movement phase, the Alien player may move up to five townsperson counters. However, these townspeople may not be:
+The Alien player moves up to five townsperson counters. These townspeople may not be:
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 -- Controlled by Town player per &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
 -- Wary per &lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
@@ -194,26 +212,11 @@
 -- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables&lt;LineBreak/&gt;
 -- Stunned per &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-In effect, the Alien player is limited to moving up to five counters that are either Alien controlled, skeptical per 
-&lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
-or totally uncontrolled. Since you are the Townsplayer, you are waiting for that to happen.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
-  </si>
-  <si>
-    <t>e003t</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e003a Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Alien player secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
-to determine which two townspersons begin the game under Alien control. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e003t Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The computer secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
-to determine which two townspersons begin the game under Alien control. This information is hidden from Towns player. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+Can move Alien controlled, skeptical per 
+&lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;, 
+or totally uncontrolled. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue006t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -613,15 +616,15 @@
         <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -648,12 +651,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="285" x14ac:dyDescent="0.25">
@@ -664,12 +667,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="225" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="240" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
started working town player movement
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\Documents\HereWeGo\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6CAD835-0B15-4E4E-B150-443C2C5FE372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{378685D3-57D2-4011-A4DF-752411AA566B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>e001</t>
   </si>
@@ -217,6 +217,21 @@
 or totally uncontrolled. Click image to continue.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue006t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e007t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e007t Town Player Movement&lt;/Bold&gt;&lt;InlineUIContainer&gt;&lt;Button Content='r6.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Town player moves any townsperson or group of townspeople in the same hex that is controlled by the Town player that are not:
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click on a green color townperson. To move a group, click on multiple townspeople in same area. Click on target area to move. If you click more than one area away, it will take a shortest random path to that location.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The alien ctonrolled counter may halt one town controlled counter from entering its space once in this phase.</t>
   </si>
 </sst>
 </file>
@@ -580,7 +595,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -675,35 +690,43 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>4</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+    <row r="16" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
working thru issues of rectangles moving
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\Documents\HereWeGo\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{378685D3-57D2-4011-A4DF-752411AA566B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1494F353-8A89-41F5-85C1-368527051DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -222,7 +222,7 @@
     <t>e007t</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e007t Town Player Movement&lt;/Bold&gt;&lt;InlineUIContainer&gt;&lt;Button Content='r6.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+    <t>&lt;Bold&gt;e007t Town Player Movement&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r6.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 The Town player moves any townsperson or group of townspeople in the same hex that is controlled by the Town player that are not:
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;

</xml_diff>

<commit_message>
starting to work Townplayer movement
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1494F353-8A89-41F5-85C1-368527051DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C7AFA8A-939A-4013-931D-C25F8E599A46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>e001</t>
   </si>
@@ -222,16 +222,28 @@
     <t>e007t</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e007t Town Player Movement&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r6.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+    <t>e008t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e007t Confirm Alien Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Confirm alien moves by clicking image.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue007t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e008t Town Player Movement&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r6.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 The Town player moves any townsperson or group of townspeople in the same hex that is controlled by the Town player that are not:
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 -- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
 -- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click on a green color townperson. To move a group, click on multiple townspeople in same area. Click on target area to move. If you click more than one area away, it will take a shortest random path to that location.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The alien ctonrolled counter may halt one town controlled counter from entering its space once in this phase.</t>
+Click on a green color townperson. To move a group, click on multiple townspeople in same area. Click on target area to move. If you click more than one area away, it will take a shortest random path to that location. When all movement is done, click on image below to continue to the next phase.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The alien controlled counter may halt all movement of one town controlled counter when it attempts to enter its space once in this phase. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue008t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -595,7 +607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -690,43 +702,51 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="180" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="210" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="B13" s="2" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    <row r="17" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
working town movement phase
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C7AFA8A-939A-4013-931D-C25F8E599A46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A70B4DBA-6324-4F31-8DBC-FD216CB74765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Events" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -241,7 +242,7 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Click on a green color townperson. To move a group, click on multiple townspeople in same area. Click on target area to move. If you click more than one area away, it will take a shortest random path to that location. When all movement is done, click on image below to continue to the next phase.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The alien controlled counter may halt all movement of one town controlled counter when it attempts to enter its space once in this phase. 
+Once in this phase, each alien controlled counter may halt all movement of one town controlled counter when it attempts to enter its space. 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue008t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>

</xml_diff>

<commit_message>
working thru influence phase
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{91B5889D-845F-446D-9854-A8ABB082E5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{FE70636A-1940-4A20-BAF1-8FAD63DF15DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>e001</t>
   </si>
@@ -249,7 +249,10 @@
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue008t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e009t Town Player Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+    <t>e010t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e009t Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Conversation is how the Town player discovers if a townsperson is Alien controlled.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -259,6 +262,18 @@
 After completion of all possible conversations, the game automatically moves to the Influence phase. Alternatively, the Town player can advance sooner by clicking image below.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue009t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e010t Infleunces&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Influencing is how the Town player convinces other uncontrolled townspeople to join their side. Click a flashing space to start a influence process.&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+To influence another uncontrolled counter, the Town player compares the Influence Factor of the Town controlled counters (bottom right per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) to the Influence Factor of the uncontrolled townsperson. The odds ration is compared to 
+&lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table, 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase. Alternatively, the Town player can advance sooner by clicking image below.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue010t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -622,7 +637,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" style="1" customWidth="1"/>
@@ -738,38 +753,46 @@
         <v>33</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="B15" s="2" t="s">
-        <v>4</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+    <row r="19" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
cleaned up unused attributes of GameInstance. Started working transition to next turn.
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE49BA37-F726-4936-BFB2-BC99D87E3E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{410DE5B3-609C-4C9B-A27E-B550D1E3D568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="16530" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>e001</t>
   </si>
@@ -252,16 +252,7 @@
     <t>e010t</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e009t Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Conversation is how the Town player discovers if a townsperson is Alien controlled.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click a flashing space to start a conversation.&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-On a roll of nine or better including modifiers from the &lt;InlineUIContainer&gt;&lt;Button Content='Conversation Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table, the Town player deteremines if it is Alien controlled counter.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-After completion of all possible conversations, the game automatically moves to the Influence phase. Alternatively, the Town player can advance sooner by clicking image below.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue009t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+    <t>e011t</t>
   </si>
   <si>
     <t>&lt;Bold&gt;e010t Influences&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
@@ -272,9 +263,40 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
 &lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase. Alternatively, the Town player can advance sooner by clicking image below.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue010t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase.</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e009t Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Conversation is how the Town player discovers if a townsperson is Alien controlled.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click a flashing space to start a conversation.&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+On a roll of nine or better including modifiers from the &lt;InlineUIContainer&gt;&lt;Button Content='Conversation Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table, the Town player deteremines if it is Alien controlled counter.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+After completion of all possible conversations, the game automatically moves to the Influence phase.</t>
+  </si>
+  <si>
+    <t>e012t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Influencing is how the Town player convinces other uncontrolled townspeople to join their side. Click a flashing space to start a influence process.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+To influence another uncontrolled counter, the Town player compares the Influence Factors (bottom right per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) and compares the odds ration to the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e011t Combats&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Influencing is how the Town player convinces other uncontrolled townspeople to join their side. Click a flashing space to start a influence process.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+To influence another uncontrolled counter, the Town player compares the Influence Factors (bottom right per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) and compares the odds ration to the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
 </sst>
 </file>
@@ -638,7 +660,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" style="1" customWidth="1"/>
@@ -749,15 +771,15 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="172.8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="144" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>35</v>
       </c>
@@ -765,35 +787,51 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+    <row r="21" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
working on takeover logic
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{410DE5B3-609C-4C9B-A27E-B550D1E3D568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45361863-CF61-4F97-9C71-60091A350F9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="16530" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -280,23 +280,17 @@
   </si>
   <si>
     <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Influencing is how the Town player convinces other uncontrolled townspeople to join their side. Click a flashing space to start a influence process.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-To influence another uncontrolled counter, the Town player compares the Influence Factors (bottom right per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) and compares the odds ration to the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e011t Combats&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Influencing is how the Town player convinces other uncontrolled townspeople to join their side. Click a flashing space to start a influence process.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-To influence another uncontrolled counter, the Town player compares the Influence Factors (bottom right per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) and compares the odds ration to the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+    <t>&lt;Bold&gt;e011t Combats&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All combat is voluntary. Combat is started by clicking a flashing red space. If the Town player attacks one or more uncontrolled counters thinking them to be Alien controlled, the result is automatically 'Attacker Wins' for the Town player, regardless of the number of uncontrolled townspeople. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Combat Factors (&lt;InlineUIContainer&gt;&lt;Button Content='r2.2.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) are compared to arriving at a postive difference (attacker is always greater number). The &lt;InlineUIContainer&gt;&lt;Button Content='Combat Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines the outcome.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;Combat can be skipped by clicking the following image.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -661,13 +655,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
   <dimension ref="A1:B21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="175.33203125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="175.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="273.60000000000002" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -675,7 +669,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -683,7 +677,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -691,7 +685,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -699,7 +693,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
@@ -707,7 +701,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -715,7 +709,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -723,7 +717,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
@@ -731,7 +725,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>23</v>
       </c>
@@ -739,7 +733,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="273.60000000000002" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -747,7 +741,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="230.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="240" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
@@ -755,7 +749,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
@@ -763,7 +757,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>31</v>
       </c>
@@ -771,7 +765,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>33</v>
       </c>
@@ -779,7 +773,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="144" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>35</v>
       </c>
@@ -787,7 +781,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>36</v>
       </c>
@@ -795,7 +789,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>39</v>
       </c>
@@ -803,7 +797,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
@@ -811,7 +805,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>3</v>
       </c>
@@ -819,7 +813,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
@@ -827,7 +821,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
started working alien and town loss tables
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B50E245C-6AB5-4CB8-9411-46D574C51BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{96B8224E-41B1-4490-88E3-438E5667E246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>e001</t>
   </si>
@@ -293,39 +293,22 @@
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue011t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
-    <t>e011aw</t>
-  </si>
-  <si>
     <t>e011af</t>
   </si>
   <si>
-    <t>e011tw</t>
-  </si>
-  <si>
     <t>e011tf</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;Bold&gt;e011aw Combats - Alien Wins&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Consult the 
- &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table. The dice are rolled for each individual counter of the defeated force, and the results are applied immediately.  </t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e011tw Combats - Town Wins&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Consult the  &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table. The dice are rolled for each individual counter of the defeated force, and the results are applied immediately.</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e011af Combats - Defender Flees&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Each counter of the must flee using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
+    <t>&lt;Bold&gt;e011af Combats - Aliens Flees&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Each counter flees using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Click image to continue.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue011af' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
     <t>&lt;Bold&gt;e011af Combats - Town Flees&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Each counter of the must flee using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
+Each counter flees using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Click image to continue.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue011tf' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
@@ -691,7 +674,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -831,70 +814,54 @@
         <v>42</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>40</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Diagnose that Shuffle of Stacks removes a stack
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{96B8224E-41B1-4490-88E3-438E5667E246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{DC18EB64-5156-40DF-ADB3-4CE30B0CEFE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -71,6 +71,227 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
+    <t>e002</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e002 Select Towns Player Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Town player rolls a die to determine which townsperson counter begins the game under his or her control according to 
+&lt;InlineUIContainer&gt;&lt;Button Content='Town Player Starting' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>e003a</t>
+  </si>
+  <si>
+    <t>e004</t>
+  </si>
+  <si>
+    <t>e005</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e001 Secretly Select HQ Area&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r3.1' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
+The Alien player secretly chooses where the Alien Sub-Commander is running his operations.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The headquarters (HQ) must be a specified building, such as &lt;Bold&gt;House 4&lt;/Bold&gt; the &lt;Bold&gt;Stock Pen&lt;/Bold&gt; , the &lt;Bold&gt;Town Hall&lt;/Bold&gt;, etc. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If the building chosen as the Alien HQ has more than one space, the Alien player must choose which area of the building is the Alien HQ. This information is secret to the Alien Player.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                       &lt;InlineUIContainer&gt;&lt;Image Name='ZebulonBlack'  Height='150' Width='150'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e004 Setting Up Map&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The starting locations for each piece is printed in the upper-left of the corner of the counter per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Every counter is placed on the map.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If a building has more than one space in it, the counter is placed randomly in one of the spaces. However, only one counter may be placed in each space. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The starting Town's controlled townsperson is shown in green. The Alien player is only one to see starting aliens until they become known. They are showed in gold. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue004' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e005 Random Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Four townspeople move randomly in any given turn. The &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines who moves. The destination is per the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Target Building' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Tied-up, Unconscious, or Killed people do not move. Stunned still move.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+If a controlled townsperson (either Town or Alien) is selected, the owner has the option to block moving it. However, the Alien player exposes that it is an alien controlled person if not known. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e006a</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e006 Alien Player Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+During his or her movement phase, the Alien player may move up to five townsperson counters. However, these townspeople may not be:
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Controlled by Town player per &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Wary per &lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables&lt;LineBreak/&gt;
+-- Stunned per &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+In effect, the Alien player is limited to moving up to five counters that are either Alien controlled, skeptical per 
+&lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
+or totally uncontrolled. Click an uncontrolled or controlled skeptical counter to move. Select their destination. They move up to their maximum movement allowance &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. You can select intermediate way points to move in a more controlled path.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click image below to continue when done moving all counters.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e005a</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e005a Awaiting Alien Confirmation of Random Move&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Alien player needs to confirm random moves before continuing.</t>
+  </si>
+  <si>
+    <t>e005t</t>
+  </si>
+  <si>
+    <t>e006t</t>
+  </si>
+  <si>
+    <t>e003t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e003a Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Alien player secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
+to determine which two townspersons begin the game under Alien control. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e003t Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The computer secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
+to determine which two townspersons begin the game under Alien control. This information is hidden from Towns player. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e005t Confirm Random Move&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Confirm random moves by clicking image.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e006t Alien Player Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Alien player moves up to five townsperson counters. These townspeople may not be:
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Controlled by Town player per &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Wary per &lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables&lt;LineBreak/&gt;
+-- Stunned per &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Can move Alien controlled, skeptical per 
+&lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;, 
+or totally uncontrolled. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue006t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e007t</t>
+  </si>
+  <si>
+    <t>e008t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e007t Confirm Alien Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Confirm alien moves by clicking image.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue007t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e009t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e008t Town Player Movement&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r6.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Town player moves any townsperson or group of townspeople in the same hex that is controlled by the Town player that are not:
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click on a green color townperson. To move a group, click on multiple townspeople in same area. Click on target area to move. If you click more than one area away, it will take a shortest random path to that location. When all movement is done, click on image below to continue to the next phase.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Once in this phase, each alien controlled counter may halt all movement of one town controlled counter when it attempts to enter its space. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue008t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e010t</t>
+  </si>
+  <si>
+    <t>e011t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e010t Influences&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Influencing is how the Town player convinces other uncontrolled townspeople to join their side. Click a flashing space to start a influence process.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+To influence another uncontrolled counter, the Town player compares the Influence Factors (bottom right per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) and compares the odds ration to the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
+&lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase.</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e009t Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Conversation is how the Town player discovers if a townsperson is Alien controlled.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click a flashing space to start a conversation.&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+On a roll of nine or better including modifiers from the &lt;InlineUIContainer&gt;&lt;Button Content='Conversation Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table, the Town player deteremines if it is Alien controlled counter.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+After completion of all possible conversations, the game automatically moves to the Influence phase.</t>
+  </si>
+  <si>
+    <t>e012t</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e011t Combats&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All combat is voluntary. Combat is started by clicking a flashing red space. If the Town player attacks one or more uncontrolled counters thinking them to be Alien controlled, the result is automatically 'Attacker Wins' for the Town player, regardless of the number of uncontrolled townspeople. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Combat Factors (&lt;InlineUIContainer&gt;&lt;Button Content='r2.2.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) are compared to arriving at a postive difference (attacker is always greater number). The &lt;InlineUIContainer&gt;&lt;Button Content='Combat Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines the outcome.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;Combat can be skipped by clicking the following image.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e011af</t>
+  </si>
+  <si>
+    <t>e011tf</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e011af Combats - Aliens Flees&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Each counter flees using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011af' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e011af Combats - Town Flees&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Each counter flees using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011tf' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
     <t>&lt;Bold&gt;e000 Game Introduction&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
 &lt;Bold&gt;They&amp;apos;ve Invaded Pleasantville&lt;/Bold&gt; minigame is a two-player game of a secret invasion by space aliens.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -80,237 +301,16 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Choose a button to begin:
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Name='ReadRules' Content=' Read Rules ' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;InlineUIContainer&gt;&lt;Button Name='ReadRules' Content=' Read Rules '  FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Rules presented as needed if choose to skip&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Name='HostGame' Content=' Host Game  ' FontFamily='Courier New'  FontSize='12'  &gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Host a game on your computer &lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Name='JoinGame' Content=' Join Game  ' FontFamily='Courier New'  FontSize='12'  &gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;InlineUIContainer&gt;&lt;Button Name='JoinGame' Content=' Join Game  '  FontFamily='Courier New'  FontSize='12'  &gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Join a game somebody is hosting&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Name='PlayTown' Content=' Town Solo  ' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Play as the Townsplayer against computer&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Name='PlayAlien' Content=' Alien Solo ' FontFamily='Courier New'  FontSize='12'  &gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
  - Play as Alien against computer&lt;LineBreak/&gt;</t>
-  </si>
-  <si>
-    <t>e002</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e002 Select Towns Player Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Town player rolls a die to determine which townsperson counter begins the game under his or her control according to 
-&lt;InlineUIContainer&gt;&lt;Button Content='Town Player Starting' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
-  </si>
-  <si>
-    <t>e003a</t>
-  </si>
-  <si>
-    <t>e004</t>
-  </si>
-  <si>
-    <t>e005</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e001 Secretly Select HQ Area&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r3.1' FontFamily='Courier New'  FontSize='12'&gt; &lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
-The Alien player secretly chooses where the Alien Sub-Commander is running his operations.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The headquarters (HQ) must be a specified building, such as &lt;Bold&gt;House 4&lt;/Bold&gt; the &lt;Bold&gt;Stock Pen&lt;/Bold&gt; , the &lt;Bold&gt;Town Hall&lt;/Bold&gt;, etc. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-If the building chosen as the Alien HQ has more than one space, the Alien player must choose which area of the building is the Alien HQ. This information is secret to the Alien Player.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                       &lt;InlineUIContainer&gt;&lt;Image Name='ZebulonBlack'  Height='150' Width='150'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e004 Setting Up Map&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The starting locations for each piece is printed in the upper-left of the corner of the counter per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Every counter is placed on the map.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-If a building has more than one space in it, the counter is placed randomly in one of the spaces. However, only one counter may be placed in each space. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The starting Town's controlled townsperson is shown in green. The Alien player is only one to see starting aliens until they become known. They are showed in gold. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue004' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e005 Random Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Four townspeople move randomly in any given turn. The &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines who moves. The destination is per the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Target Building' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Tied-up, Unconscious, or Killed people do not move. Stunned still move.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-If a controlled townsperson (either Town or Alien) is selected, the owner has the option to block moving it. However, the Alien player exposes that it is an alien controlled person if not known. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>e006a</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e006 Alien Player Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-During his or her movement phase, the Alien player may move up to five townsperson counters. However, these townspeople may not be:
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
--- Controlled by Town player per &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
--- Wary per &lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
--- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
--- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables&lt;LineBreak/&gt;
--- Stunned per &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-In effect, the Alien player is limited to moving up to five counters that are either Alien controlled, skeptical per 
-&lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
-or totally uncontrolled. Click an uncontrolled or controlled skeptical counter to move. Select their destination. They move up to their maximum movement allowance &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. You can select intermediate way points to move in a more controlled path.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click image below to continue when done moving all counters.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>e005a</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e005a Awaiting Alien Confirmation of Random Move&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Alien player needs to confirm random moves before continuing.</t>
-  </si>
-  <si>
-    <t>e005t</t>
-  </si>
-  <si>
-    <t>e006t</t>
-  </si>
-  <si>
-    <t>e003t</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e003a Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Alien player secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
-to determine which two townspersons begin the game under Alien control. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e003t Roll for Alien Controlled Counter&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The computer secretly rolls the dice twice on the &lt;InlineUIContainer&gt;&lt;Button Content='Townspeople' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table 
-to determine which two townspersons begin the game under Alien control. This information is hidden from Towns player. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                       &lt;InlineUIContainer&gt;&lt;Image Name='Continue003a' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e005t Confirm Random Move&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Confirm random moves by clicking image.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e006t Alien Player Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Alien player moves up to five townsperson counters. These townspeople may not be:
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
--- Controlled by Town player per &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
--- Wary per &lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
--- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
--- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables&lt;LineBreak/&gt;
--- Stunned per &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Can move Alien controlled, skeptical per 
-&lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;, 
-or totally uncontrolled. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue006t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>e007t</t>
-  </si>
-  <si>
-    <t>e008t</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e007t Confirm Alien Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Confirm alien moves by clicking image.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue007t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>e009t</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e008t Town Player Movement&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r6.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Town player moves any townsperson or group of townspeople in the same hex that is controlled by the Town player that are not:
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
--- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
--- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click on a green color townperson. To move a group, click on multiple townspeople in same area. Click on target area to move. If you click more than one area away, it will take a shortest random path to that location. When all movement is done, click on image below to continue to the next phase.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Once in this phase, each alien controlled counter may halt all movement of one town controlled counter when it attempts to enter its space. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue008t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>e010t</t>
-  </si>
-  <si>
-    <t>e011t</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e010t Influences&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Influencing is how the Town player convinces other uncontrolled townspeople to join their side. Click a flashing space to start a influence process.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-To influence another uncontrolled counter, the Town player compares the Influence Factors (bottom right per &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) and compares the odds ration to the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Influence Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table adjusting with the 
-&lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-After completion of all possible infleunces have occurred, the game automatically moves to the Combat phase.</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e009t Conversations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Conversation is how the Town player discovers if a townsperson is Alien controlled.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click a flashing space to start a conversation.&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-On a roll of nine or better including modifiers from the &lt;InlineUIContainer&gt;&lt;Button Content='Conversation Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table, the Town player deteremines if it is Alien controlled counter.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-After completion of all possible conversations, the game automatically moves to the Influence phase.</t>
-  </si>
-  <si>
-    <t>e012t</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e011t Combats&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-All combat is voluntary. Combat is started by clicking a flashing red space. If the Town player attacks one or more uncontrolled counters thinking them to be Alien controlled, the result is automatically 'Attacker Wins' for the Town player, regardless of the number of uncontrolled townspeople. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Combat Factors (&lt;InlineUIContainer&gt;&lt;Button Content='r2.2.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;) are compared to arriving at a postive difference (attacker is always greater number). The &lt;InlineUIContainer&gt;&lt;Button Content='Combat Results' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table determines the outcome.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;Combat can be skipped by clicking the following image.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>e011af</t>
-  </si>
-  <si>
-    <t>e011tf</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e011af Combats - Aliens Flees&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Each counter flees using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011af' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e011af Combats - Town Flees&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Each counter flees using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011tf' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -686,7 +686,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -694,143 +694,143 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="240" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
working limiting town stacking
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BDE52F4-0551-480A-99BD-589CFDE70531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9CE5D485-7DD5-4D04-9C5D-E9C86AFE2252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>e001</t>
   </si>
@@ -111,25 +111,6 @@
   </si>
   <si>
     <t>e006a</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e006 Alien Player Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-During his or her movement phase, the Alien player may move up to five townsperson counters. However, these townspeople may not be:
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
--- Controlled by Town player per &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
--- Wary per &lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
--- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
--- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables&lt;LineBreak/&gt;
--- Stunned per &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-In effect, the Alien player is limited to moving up to five counters that are either Alien controlled, skeptical per 
-&lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
-or totally uncontrolled. Click an uncontrolled or controlled skeptical counter to move. Select their destination. They move up to their maximum movement allowance &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. You can select intermediate way points to move in a more controlled path.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click image below to continue when done moving all counters.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
     <t>e005a</t>
@@ -291,20 +272,6 @@
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='128'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e012t.1 Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The alien sub-commander, Zebulon, is not discovered. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue012t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e012t.2 Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Since Town player guessed the correct location, the Alien sub-commander, Zebulon, is placed on the map board. The Town player can win by engaging and defeating Zebulon in combat. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue012t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
     <t>e012t1</t>
   </si>
   <si>
@@ -337,14 +304,61 @@
                                 &lt;InlineUIContainer&gt;&lt;Image Name='Alien' Height='100' Width='130'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
+    <t>&lt;Bold&gt;e012t1 Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The alien sub-commander, Zebulon, is not discovered. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue012t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e012t2 Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Since Town player guessed the correct location, the Alien sub-commander, Zebulon, is placed on the map board. The Town player can win by engaging and defeating Zebulon in combat. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue012t' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e006a Alien Player Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+During his or her movement phase, the Alien player may move up to five townsperson counters. However, these townspeople may not be:
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Controlled by Town player per &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Wary per &lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
+-- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables&lt;LineBreak/&gt;
+-- Stunned per &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+In effect, the Alien player is limited to moving up to five counters that are either Alien controlled, skeptical per 
+&lt;InlineUIContainer&gt;&lt;Button Content='r7.2.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
+or totally uncontrolled. Click an uncontrolled or controlled skeptical counter to move. Select their destination. They move up to their maximum movement allowance &lt;InlineUIContainer&gt;&lt;Button Content='r5.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. You can select intermediate way points to move in a more controlled path.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click image below to continue when done moving all counters.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue005' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e008t1</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e008t1 Town Player Movement - Overstacking&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r6.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+The Town player are overstacked in the flashing spaces. The town player must move counters away from these spaces to reduce the number of controlled town controlled counters to three.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click on a green color townperson. Click on target area to move. If you click more than one area away, it takes a shortest random path to that location.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Once in this phase, each alien controlled counter may halt all movement of one town controlled counter when it attempts to enter its space. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
     <t>&lt;Bold&gt;e008t Town Player Movement&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r6.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
-The Town player moves any townsperson or group of townspeople in the same hex that is controlled by the Town player that are not:
+The Town player moves any townsperson controlled by the Town player that are not:
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 -- Tied Up per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;&lt;LineBreak/&gt;
 -- Unconscious per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click on a green color townperson. To move a group, click on multiple townspeople in same area. Click on target area to move. If you click more than one area away, it takes a shortest random path to that location.
+-- Stunned per &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; or &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Tables
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click on a green color townperson. Click on target area to move. If you click more than one area away, it takes a shortest random path to that location.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Once in this phase, each alien controlled counter may halt all movement of one town controlled counter when it attempts to enter its space. 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -714,7 +728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -726,7 +740,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -750,15 +764,15 @@
         <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -774,23 +788,23 @@
         <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="285" x14ac:dyDescent="0.25">
@@ -798,134 +812,142 @@
         <v>17</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="240" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="255" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="240" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="135" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="150" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="165" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="90" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="120" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B26" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+    <row r="27" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
working town player move
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9CE5D485-7DD5-4D04-9C5D-E9C86AFE2252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2655F6DC-C626-43FF-92B8-F85BFF79DF74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="28680" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>e001</t>
   </si>
@@ -207,13 +207,6 @@
 Each counter flees using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Click image to continue.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                         &lt;InlineUIContainer&gt;&lt;Image Name='Continue011af' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Bold&gt;e011af Combats - Town Flees&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Each counter flees using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011tf' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
     <t>&lt;Bold&gt;e000 Game Introduction&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt; 
@@ -365,6 +358,22 @@
 When all movement is done, click on image below to continue to the next phase.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                               &lt;InlineUIContainer&gt;&lt;Image Name='Welcome' Height='125' Width='200'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>e011ts</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e011tf Combats - Town Flees&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Each counter flees using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                        &lt;InlineUIContainer&gt;&lt;Image Name='Continue011tf' Height='100' Width='100'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e011ts Combats - Town Counter Stunned&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Stunned town people retreat one space. Click on one of the blue colored spaces to retreat the town player counter.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
 </sst>
 </file>
@@ -728,7 +737,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F7370C4-35CC-4CF6-93A4-4A91468DAED0}">
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="1" customWidth="1"/>
@@ -740,7 +749,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -788,7 +797,7 @@
         <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -812,7 +821,7 @@
         <v>17</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -820,7 +829,7 @@
         <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -836,15 +845,15 @@
         <v>27</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -868,7 +877,7 @@
         <v>31</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -884,70 +893,78 @@
         <v>36</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="B21" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="90" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="120" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+    <row r="28" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
do not show die when doing observations
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2655F6DC-C626-43FF-92B8-F85BFF79DF74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE4854B9-3660-4CDE-A10A-4EBC7F3F007D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="5700" yWindow="2355" windowWidth="21600" windowHeight="11145" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Events" sheetId="1" r:id="rId1"/>
@@ -271,15 +271,6 @@
     <t>e012t2</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Any conscious, defeated, Alien controlled counter may be interrogated by a Town controlled piece. Choose a building area that is not colored black. If Zebulon is found, the counter is placed on the board and can be defeated in combat to win the game. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click a flashing space to begin.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                    &lt;InlineUIContainer&gt;&lt;Image Name='Interrogation' Height='180' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;e006t Alien Player Movement&lt;/Bold&gt; &lt;InlineUIContainer&gt;&lt;Button Content='r6.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 The Alien player moves up to five townsperson counters. These townspeople may not be:
@@ -374,6 +365,15 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Stunned town people retreat one space. Click on one of the blue colored spaces to retreat the town player counter.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e012t Interrogations&lt;/Bold&gt;  &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Any conscious, defeated, Alien controlled counter may be interrogated by a Town controlled piece. Choose a building area that is not colored black. If Zebulon is found, the counter is placed on the board and can be defeated in combat to win the game. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click a flashing space to begin.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                &lt;InlineUIContainer&gt;&lt;Image Name='Interrogation' Height='180' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -821,7 +821,7 @@
         <v>17</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -829,7 +829,7 @@
         <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -845,15 +845,15 @@
         <v>27</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -893,15 +893,15 @@
         <v>36</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -909,7 +909,7 @@
         <v>34</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -917,7 +917,7 @@
         <v>43</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -925,7 +925,7 @@
         <v>44</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="120" x14ac:dyDescent="0.25">

</xml_diff>